<commit_message>
resolved main and plot issues
</commit_message>
<xml_diff>
--- a/reconcile/storage/input/zev_og_clean.xlsx
+++ b/reconcile/storage/input/zev_og_clean.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T45"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,10 +525,15 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>capacity_id</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>project_key_str</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>project_key_tuple</t>
         </is>
@@ -615,10 +620,15 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
+          <t>prod_DB_9aa81188-d35f-5bf6-b760-44b1f80b4d6c_27777.777777777777</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>DE|Leipzig|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>('DE', 'Leipzig', "('bmw',)", 'vehicle')</t>
         </is>
@@ -705,10 +715,15 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
+          <t>prod_DB_9aa81188-d35f-5bf6-b760-44b1f80b4d6c_100000.0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>DE|Leipzig|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>('DE', 'Leipzig', "('bmw',)", 'vehicle')</t>
         </is>
@@ -799,10 +814,15 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
+          <t>prod_DB_655601d6-44d7-5fae-9f00-aed5f36c0462_20016.0</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>DE|Munich|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>('DE', 'Munich', "('bmw',)", 'vehicle')</t>
         </is>
@@ -891,10 +911,15 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
+          <t>prod_DB_655601d6-44d7-5fae-9f00-aed5f36c0462_nan</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
           <t>DE|Munich|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>('DE', 'Munich', "('bmw',)", 'vehicle')</t>
         </is>
@@ -985,10 +1010,15 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
+          <t>prod_DB_6d0da839-f19a-5497-8a1f-befe19c9e09b_113031.93000000001</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
           <t>DE|Regensburg|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>('DE', 'Regensburg', "('bmw',)", 'vehicle')</t>
         </is>
@@ -1079,10 +1109,15 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
+          <t>prod_DB_6d0da839-f19a-5497-8a1f-befe19c9e09b_156831.93</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
           <t>DE|Regensburg|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>('DE', 'Regensburg', "('bmw',)", 'vehicle')</t>
         </is>
@@ -1169,10 +1204,15 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
+          <t>prod_DB_1fba0998-ffe7-54f5-a236-919e234e7829_46387.0</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>GB|Oxfordshire|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>('GB', 'Oxfordshire', "('bmw',)", 'vehicle')</t>
         </is>
@@ -1243,10 +1283,15 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
+          <t>prod_DB_ecd072cf-0eac-532c-9197-9ec57c2ffeb7_1076.0</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
           <t>GB|None|('bmw',)|vehicle</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>('GB', 'None', "('bmw',)", 'vehicle')</t>
         </is>
@@ -1335,10 +1380,15 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
+          <t>prod_DB_a6afa10f-a63b-5eac-88f5-91a2fe0c95f2_nan</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
           <t>GB|Oxfordshire|('arrival',)|vehicle</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>('GB', 'Oxfordshire', "('arrival',)", 'vehicle')</t>
         </is>
@@ -1425,10 +1475,15 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
+          <t>prod_DB_d005f306-6f24-5243-9c14-757b40e8e259_50339.0</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
           <t>BE|Arrondissement Brussel-Hoofdstad|('audi',)|vehicle</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>('BE', 'Arrondissement Brussel-Hoofdstad', "('audi',)", 'vehicle')</t>
         </is>
@@ -1519,10 +1574,15 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
+          <t>prod_DB_f3187b2a-14b8-5526-ac0e-fa9f6dc48897_15411.0</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
           <t>DE|Ingolstadt|('audi',)|vehicle</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>('DE', 'Ingolstadt', "('audi',)", 'vehicle')</t>
         </is>
@@ -1613,10 +1673,15 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
+          <t>prod_DB_8c10f625-fea2-51ad-a118-adb9ac7fbea1_28334.0</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
           <t>DE|Neckarsulm|('audi',)|vehicle</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>('DE', 'Neckarsulm', "('audi',)", 'vehicle')</t>
         </is>
@@ -1685,10 +1750,15 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
+          <t>prod_DB_22ff6ad3-2641-5943-8217-7da301746c58_nan</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
           <t>FR|None|('byd',)|vehicle</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>('FR', 'None', "('byd',)", 'vehicle')</t>
         </is>
@@ -1767,10 +1837,15 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
+          <t>prod_DB_87ed39d0-95e7-55f0-9c84-367ea52968ab_400.0</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
           <t>HU|Komárom-Esztergom|('byd',)|vehicle</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>('HU', 'Komárom-Esztergom', "('byd',)", 'vehicle')</t>
         </is>
@@ -1861,10 +1936,15 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
+          <t>prod_DB_0ec09a24-125b-5eee-a2c2-db6f7c89e362_250000.0</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
           <t>DE|Cologne|('ford',)|vehicle</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>('DE', 'Cologne', "('ford',)", 'vehicle')</t>
         </is>
@@ -1951,10 +2031,15 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
+          <t>prod_DB_91c3a3a6-5ae4-5816-bdb3-9af8631e0671_72052.0</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
           <t>CZ|Nošovice|('hyundai',)|vehicle</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="U17" t="inlineStr">
         <is>
           <t>('CZ', 'Nošovice', "('hyundai',)", 'vehicle')</t>
         </is>
@@ -2041,10 +2126,15 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
+          <t>prod_DB_7a65fbfe-29d4-5f10-95e3-8cf4634b0088_37239.0</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
           <t>SK|Žilina Region|('kia',)|vehicle</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr">
+      <c r="U18" t="inlineStr">
         <is>
           <t>('SK', 'Žilina Region', "('kia',)", 'vehicle')</t>
         </is>
@@ -2131,10 +2221,15 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
+          <t>prod_DB_303ad2bc-a853-55e8-9566-858510f8d770_18427.0</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
           <t>DE|Bremen|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="U19" t="inlineStr">
         <is>
           <t>('DE', 'Bremen', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2205,10 +2300,15 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
+          <t>prod_DB_5adfe1a0-5af6-579e-b8fc-45382ca79c99_4760.0</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
           <t>DE|None|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="U20" t="inlineStr">
         <is>
           <t>('DE', 'None', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2277,10 +2377,15 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
+          <t>prod_DB_5adfe1a0-5af6-579e-b8fc-45382ca79c99_nan</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
           <t>DE|None|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>('DE', 'None', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2371,10 +2476,15 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
+          <t>prod_DB_728fcd34-e11b-59cc-ac72-f6f4bfd53540_83195.0</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
           <t>DE|Rastatt|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T22" t="inlineStr">
+      <c r="U22" t="inlineStr">
         <is>
           <t>('DE', 'Rastatt', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2465,10 +2575,15 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
+          <t>prod_DB_1a71a177-e936-50c5-9103-940e7397cc66_62577.5</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
           <t>DE|Sindelfingen|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="U23" t="inlineStr">
         <is>
           <t>('DE', 'Sindelfingen', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2539,10 +2654,15 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
+          <t>prod_DB_c1ab1fd2-af88-5319-8d29-f5f844946c36_10739.0</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
           <t>ES|None|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>('ES', 'None', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2621,10 +2741,15 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
+          <t>prod_DB_792aa593-f545-506e-876a-c8156d0c4131_50444.0</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
           <t>HU|Bács-Kiskun|('mercedes benz',)|vehicle</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="U25" t="inlineStr">
         <is>
           <t>('HU', 'Bács-Kiskun', "('mercedes benz',)", 'vehicle')</t>
         </is>
@@ -2707,10 +2832,15 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
+          <t>prod_DB_f119dc73-a41d-541d-96ec-a7f18a74dcab_40710.0</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
           <t>GB|Sunderland|('nissan',)|vehicle</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="U26" t="inlineStr">
         <is>
           <t>('GB', 'Sunderland', "('nissan',)", 'vehicle')</t>
         </is>
@@ -2791,10 +2921,15 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
+          <t>prod_DB_916f228d-de7f-5acb-9645-66e4b8495022_nan</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
           <t>HR|Krapina-Zagorje|('rimac automobili',)|vehicle</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="U27" t="inlineStr">
         <is>
           <t>('HR', 'Krapina-Zagorje', "('rimac automobili',)", 'vehicle')</t>
         </is>
@@ -2881,10 +3016,15 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
+          <t>prod_DB_f2de5535-0d2e-5fe4-971b-d70bcab45f62_20135.0</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
           <t>ES|Catalonia|('seat',)|vehicle</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="U28" t="inlineStr">
         <is>
           <t>('ES', 'Catalonia', "('seat',)", 'vehicle')</t>
         </is>
@@ -2971,10 +3111,15 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
+          <t>prod_DB_69a8d694-a8ef-5977-9cb4-95e721a1c2b5_79507.0</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
           <t>CZ|Mladá Boleslav|('skoda',)|vehicle</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>('CZ', 'Mladá Boleslav', "('skoda',)", 'vehicle')</t>
         </is>
@@ -3059,10 +3204,15 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
+          <t>prod_DB_69a8d694-a8ef-5977-9cb4-95e721a1c2b5_nan</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
           <t>CZ|Mladá Boleslav|('skoda',)|vehicle</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr">
+      <c r="U30" t="inlineStr">
         <is>
           <t>('CZ', 'Mladá Boleslav', "('skoda',)", 'vehicle')</t>
         </is>
@@ -3149,10 +3299,15 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
+          <t>prod_DB_b4cab349-dacc-5f73-8e7b-483f322893e7_9653.0</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
           <t>DE|Eisenach|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="U31" t="inlineStr">
         <is>
           <t>('DE', 'Eisenach', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3237,10 +3392,15 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
+          <t>prod_DB_b4cab349-dacc-5f73-8e7b-483f322893e7_nan</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
           <t>DE|Eisenach|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="U32" t="inlineStr">
         <is>
           <t>('DE', 'Eisenach', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3327,10 +3487,15 @@
       </c>
       <c r="S33" t="inlineStr">
         <is>
+          <t>prod_DB_3d932cba-5ffc-5a17-b4c0-f20c2d5ba0b5_49264.0</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
           <t>SK|Trnava Region|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
+      <c r="U33" t="inlineStr">
         <is>
           <t>('SK', 'Trnava Region', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3415,10 +3580,15 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
+          <t>prod_DB_3d932cba-5ffc-5a17-b4c0-f20c2d5ba0b5_nan</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
           <t>SK|Trnava Region|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="U34" t="inlineStr">
         <is>
           <t>('SK', 'Trnava Region', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3505,10 +3675,15 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
+          <t>prod_DB_408c902f-cfa7-504a-9977-6439e267cf6f_3734.0</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
           <t>ES|Galicia|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="U35" t="inlineStr">
         <is>
           <t>('ES', 'Galicia', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3593,10 +3768,15 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
+          <t>prod_DB_408c902f-cfa7-504a-9977-6439e267cf6f_nan</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
           <t>ES|Galicia|('stellantis',)|vehicle</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="U36" t="inlineStr">
         <is>
           <t>('ES', 'Galicia', "('stellantis',)", 'vehicle')</t>
         </is>
@@ -3683,10 +3863,15 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
+          <t>prod_DB_ab942289-b19a-5128-8112-1c5a42e60372_206097.0</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
           <t>DE|Berlin|('tesla',)|vehicle</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>('DE', 'Berlin', "('tesla',)", 'vehicle')</t>
         </is>
@@ -3767,10 +3952,15 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
+          <t>prod_DB_868eec56-32a9-5703-bb1c-5381dda72cb9_nan</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
           <t>NL|Tilburg Municipality|('tesla',)|vehicle</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="U38" t="inlineStr">
         <is>
           <t>('NL', 'Tilburg Municipality', "('tesla',)", 'vehicle')</t>
         </is>
@@ -3849,10 +4039,15 @@
       </c>
       <c r="S39" t="inlineStr">
         <is>
+          <t>prod_DB_24f54170-5f2a-500a-8994-da2daf36ed6a_94839.0</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
           <t>SK|Bratislava Region|('volkswagen',)|vehicle</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>('SK', 'Bratislava Region', "('volkswagen',)", 'vehicle')</t>
         </is>
@@ -3939,10 +4134,15 @@
       </c>
       <c r="S40" t="inlineStr">
         <is>
+          <t>prod_DB_5407b64f-8759-5926-9898-d6b7600bdfe1_333000.0</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
           <t>DE|Zwickau|('volkswagen',)|vehicle</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="U40" t="inlineStr">
         <is>
           <t>('DE', 'Zwickau', "('volkswagen',)", 'vehicle')</t>
         </is>
@@ -4011,10 +4211,15 @@
       </c>
       <c r="S41" t="inlineStr">
         <is>
+          <t>prod_DB_1e021201-2d98-52e5-9905-7ccb21bf9a34_nan</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
           <t>FR|None|('volvo group',)|vehicle</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="U41" t="inlineStr">
         <is>
           <t>('FR', 'None', "('volvo group',)", 'vehicle')</t>
         </is>
@@ -4103,10 +4308,15 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
+          <t>prod_DB_bcdccb94-69aa-5c33-a476-6cd3838c0c57_nan</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
           <t>BE|Arrondissement of Ghent|('volvo group',)|vehicle</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="U42" t="inlineStr">
         <is>
           <t>('BE', 'Arrondissement of Ghent', "('volvo group',)", 'vehicle')</t>
         </is>
@@ -4195,10 +4405,15 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
+          <t>prod_DB_bcdccb94-69aa-5c33-a476-6cd3838c0c57_nan</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
           <t>BE|Arrondissement of Ghent|('volvo group',)|vehicle</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="U43" t="inlineStr">
         <is>
           <t>('BE', 'Arrondissement of Ghent', "('volvo group',)", 'vehicle')</t>
         </is>
@@ -4283,10 +4498,15 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
+          <t>prod_DB_43827abe-ea8c-5a39-87d9-c1114db92c51_nan</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
           <t>SE|Västra Götaland|('volvo',)|vehicle</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr">
+      <c r="U44" t="inlineStr">
         <is>
           <t>('SE', 'Västra Götaland', "('volvo',)", 'vehicle')</t>
         </is>
@@ -4373,10 +4593,15 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
+          <t>prod_DB_e2b88591-16ed-593d-81d0-f4437853d855_14287.0</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
           <t>GB|Knowsley|('tata jlr',)|vehicle</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr">
+      <c r="U45" t="inlineStr">
         <is>
           <t>('GB', 'Knowsley', "('tata jlr',)", 'vehicle')</t>
         </is>

</xml_diff>

<commit_message>
ev volumes from main
</commit_message>
<xml_diff>
--- a/reconcile/storage/input/zev_og_clean.xlsx
+++ b/reconcile/storage/input/zev_og_clean.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V54"/>
+  <dimension ref="A1:V56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3104,7 +3104,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -3113,11 +3113,11 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>45657</v>
+        <v>40908</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_ae2d47e1-87d3-57a5-a054-c96dec440280_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_ae2d47e1-87d3-57a5-a054-c96dec440280_20000.0</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3194,12 +3194,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>batilly</t>
+          <t>maubeuge</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>batilly</t>
+          <t>maubeuge</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -3217,11 +3217,11 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>expansion</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>45657</v>
+        <v>45291</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -3235,34 +3235,34 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Batilly</t>
+          <t>Maubeuge</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Grand Est</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Meurthe et Moselle</t>
+          <t>North</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Arrondissement of Briey</t>
+          <t>Arrondissement of Avesnes-sur-Helpe</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Batilly</t>
+          <t>Maubeuge</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>49.17372</v>
+        <v>50.27875</v>
       </c>
       <c r="Q29" t="n">
-        <v>5.96869</v>
+        <v>3.97267</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -3271,22 +3271,22 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>307c4123-5be8-5174-ad9d-1840e75df719</t>
+          <t>ae2d47e1-87d3-57a5-a054-c96dec440280</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_307c4123-5be8-5174-ad9d-1840e75df719_0.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_ae2d47e1-87d3-57a5-a054-c96dec440280_40000.0</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>FR|Batilly|renault|vehicle</t>
+          <t>FR|Maubeuge|renault|vehicle</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>('FR', 'Batilly', 'renault', 'vehicle')</t>
+          <t>('FR', 'Maubeuge', 'renault', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -3298,12 +3298,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>sandouville</t>
+          <t>batilly</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sandouville</t>
+          <t>batilly</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3325,7 +3325,7 @@
         </is>
       </c>
       <c r="H30" s="2" t="n">
-        <v>45657</v>
+        <v>43830</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -3339,34 +3339,34 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Sandouville</t>
+          <t>Batilly</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Normandy</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Seine-Maritime</t>
+          <t>Meurthe et Moselle</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Arrondissement of Le Havre</t>
+          <t>Arrondissement of Briey</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Sandouville</t>
+          <t>Batilly</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>49.4978</v>
+        <v>49.17372</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.31748</v>
+        <v>5.96869</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -3375,22 +3375,22 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>424b7ed5-fc12-5e41-b341-a5b1dde327f5</t>
+          <t>307c4123-5be8-5174-ad9d-1840e75df719</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_424b7ed5-fc12-5e41-b341-a5b1dde327f5_0.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_307c4123-5be8-5174-ad9d-1840e75df719_0.0</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>FR|Sandouville|renault|vehicle</t>
+          <t>FR|Batilly|renault|vehicle</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>('FR', 'Sandouville', 'renault', 'vehicle')</t>
+          <t>('FR', 'Batilly', 'renault', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>80000</v>
+        <v>120000</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -3425,11 +3425,11 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
-        <v>44561</v>
+        <v>44926</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_252dc9b3-ab0a-55e9-873c-064f96c53ea6_80000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_252dc9b3-ab0a-55e9-873c-064f96c53ea6_120000.0</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3506,12 +3506,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>douai</t>
+          <t>flins</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>douai</t>
+          <t>flins</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -3529,11 +3529,11 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>expansion</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
-        <v>45657</v>
+        <v>41639</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -3547,34 +3547,34 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Douai</t>
+          <t>Flins-sur-Seine</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Yvelines</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Arrondissement of Douai</t>
+          <t>Arrondissement of Mantes-la-Jolie</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Douai</t>
+          <t>Flins-sur-Seine</t>
         </is>
       </c>
       <c r="P32" t="n">
-        <v>50.37069</v>
+        <v>48.96523</v>
       </c>
       <c r="Q32" t="n">
-        <v>3.07922</v>
+        <v>1.87314</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -3583,22 +3583,22 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>252dc9b3-ab0a-55e9-873c-064f96c53ea6</t>
+          <t>5140a707-9f43-506f-868e-0bce2129328e</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_252dc9b3-ab0a-55e9-873c-064f96c53ea6_120000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_5140a707-9f43-506f-868e-0bce2129328e_80000.0</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>FR|Douai|renault|vehicle</t>
+          <t>FR|Flins-sur-Seine|renault|vehicle</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>('FR', 'Douai', 'renault', 'vehicle')</t>
+          <t>('FR', 'Flins-sur-Seine', 'renault', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>40000</v>
+        <v>160000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -3633,11 +3633,11 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>expansion</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
-        <v>45291</v>
+        <v>44196</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_5140a707-9f43-506f-868e-0bce2129328e_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_5140a707-9f43-506f-868e-0bce2129328e_160000.0</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3714,21 +3714,21 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>novo mesto</t>
+          <t>flins</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>novo_mesto</t>
+          <t>flins</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -3737,11 +3737,11 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>greenfield</t>
+          <t>expansion</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
-        <v>44196</v>
+        <v>45657</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -3755,22 +3755,34 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Novo Mesto</t>
+          <t>Flins-sur-Seine</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Novo Mesto</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Yvelines</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Arrondissement of Mantes-la-Jolie</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Flins-sur-Seine</t>
+        </is>
+      </c>
       <c r="P34" t="n">
-        <v>45.80397</v>
+        <v>48.96523</v>
       </c>
       <c r="Q34" t="n">
-        <v>15.16886</v>
+        <v>1.87314</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -3779,48 +3791,48 @@
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>cae893de-e792-5121-b6a8-75f1cf517027</t>
+          <t>5140a707-9f43-506f-868e-0bce2129328e</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_cae893de-e792-5121-b6a8-75f1cf517027_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_5140a707-9f43-506f-868e-0bce2129328e_0.0</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>SI|Novo Mesto|renault|vehicle</t>
+          <t>FR|Flins-sur-Seine|renault|vehicle</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>('SI', 'Novo Mesto', 'renault', 'vehicle')</t>
+          <t>('FR', 'Flins-sur-Seine', 'renault', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>seat</t>
+          <t>renault</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>martorell</t>
+          <t>novo mesto</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>martorell</t>
+          <t>novo_mesto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>80000</v>
+        <v>40000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -3833,7 +3845,7 @@
         </is>
       </c>
       <c r="H35" s="2" t="n">
-        <v>44197</v>
+        <v>44196</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -3847,30 +3859,22 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Martorell</t>
+          <t>Novo Mesto</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Catalonia</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Barcelona</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Martorell</t>
-        </is>
-      </c>
+          <t>Novo Mesto</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="n">
-        <v>41.47402</v>
+        <v>45.80397</v>
       </c>
       <c r="Q35" t="n">
-        <v>1.93062</v>
+        <v>15.16886</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -3879,48 +3883,48 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>fd4bfcba-5859-5681-a582-2f56b17afe5d</t>
+          <t>cae893de-e792-5121-b6a8-75f1cf517027</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_fd4bfcba-5859-5681-a582-2f56b17afe5d_80000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_cae893de-e792-5121-b6a8-75f1cf517027_40000.0</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>ES|Martorell|seat|vehicle</t>
+          <t>SI|Novo Mesto|renault|vehicle</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>('ES', 'Martorell', 'seat', 'vehicle')</t>
+          <t>('SI', 'Novo Mesto', 'renault', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>skoda</t>
+          <t>seat</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>mladá boleslav</t>
+          <t>martorell</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>mladá_boleslav</t>
+          <t>martorell</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>120000</v>
+        <v>80000</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -3933,7 +3937,7 @@
         </is>
       </c>
       <c r="H36" s="2" t="n">
-        <v>44075</v>
+        <v>44197</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -3947,30 +3951,30 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Mladá Boleslav</t>
+          <t>Martorell</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Central Bohemia</t>
+          <t>Catalonia</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Mladá Boleslav District</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Mladá Boleslav</t>
+          <t>Martorell</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="n">
-        <v>50.41135</v>
+        <v>41.47402</v>
       </c>
       <c r="Q36" t="n">
-        <v>14.90318</v>
+        <v>1.93062</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -3979,61 +3983,61 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>f1bee7e3-ba81-5e19-b58b-196acd14eee5</t>
+          <t>fd4bfcba-5859-5681-a582-2f56b17afe5d</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_f1bee7e3-ba81-5e19-b58b-196acd14eee5_120000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_fd4bfcba-5859-5681-a582-2f56b17afe5d_80000.0</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>CZ|Mladá Boleslav|skoda|vehicle</t>
+          <t>ES|Martorell|seat|vehicle</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>('CZ', 'Mladá Boleslav', 'skoda', 'vehicle')</t>
+          <t>('ES', 'Martorell', 'seat', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>stellantis</t>
+          <t>skoda</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>poissy</t>
+          <t>mladá boleslav</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>poissy</t>
+          <t>mladá_boleslav</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>40000</v>
+        <v>120000</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>operational</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">
-        <v>45291</v>
+        <v>44075</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -4047,34 +4051,30 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Poissy</t>
+          <t>Mladá Boleslav</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Central Bohemia</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Yvelines</t>
+          <t>Mladá Boleslav District</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Arrondissement of Saint-Germain-en-Laye</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Poissy</t>
-        </is>
-      </c>
+          <t>Mladá Boleslav</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="n">
-        <v>48.92902</v>
+        <v>50.41135</v>
       </c>
       <c r="Q37" t="n">
-        <v>2.04952</v>
+        <v>14.90318</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -4083,22 +4083,22 @@
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1a826860-cc3f-5c7d-9e41-ab9563a927fc</t>
+          <t>f1bee7e3-ba81-5e19-b58b-196acd14eee5</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_1a826860-cc3f-5c7d-9e41-ab9563a927fc_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_f1bee7e3-ba81-5e19-b58b-196acd14eee5_120000.0</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>FR|Poissy|stellantis|vehicle</t>
+          <t>CZ|Mladá Boleslav|skoda|vehicle</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>('FR', 'Poissy', 'stellantis', 'vehicle')</t>
+          <t>('CZ', 'Mladá Boleslav', 'skoda', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -4110,20 +4110,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>vigo</t>
+          <t>poissy</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>vigo</t>
+          <t>poissy</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>40000</v>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>operational</t>
@@ -4131,11 +4133,11 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>expansion</t>
+          <t>retrofit</t>
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>44502</v>
+        <v>44561</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -4149,30 +4151,34 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Vigo</t>
+          <t>Poissy</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Galicia</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Pontevedra</t>
+          <t>Yvelines</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Vigo</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr"/>
+          <t>Arrondissement of Saint-Germain-en-Laye</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Poissy</t>
+        </is>
+      </c>
       <c r="P38" t="n">
-        <v>42.23282</v>
+        <v>48.92902</v>
       </c>
       <c r="Q38" t="n">
-        <v>-8.72264</v>
+        <v>2.04952</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -4181,22 +4187,22 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>5ffe50f9-d148-5c9a-9d53-5afd17293ea1</t>
+          <t>1a826860-cc3f-5c7d-9e41-ab9563a927fc</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_5ffe50f9-d148-5c9a-9d53-5afd17293ea1_nan</t>
+          <t>68d684fc1c2e9d8ed1487afa_1a826860-cc3f-5c7d-9e41-ab9563a927fc_40000.0</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>ES|Vigo|stellantis|vehicle</t>
+          <t>FR|Poissy|stellantis|vehicle</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>('ES', 'Vigo', 'stellantis', 'vehicle')</t>
+          <t>('FR', 'Poissy', 'stellantis', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4328,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>80000</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -4335,7 +4341,7 @@
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>41061</v>
+        <v>44562</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -4386,7 +4392,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_5ffe50f9-d148-5c9a-9d53-5afd17293ea1_0.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_5ffe50f9-d148-5c9a-9d53-5afd17293ea1_80000.0</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
@@ -4435,7 +4441,7 @@
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>43831</v>
+        <v>45658</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -4730,16 +4736,16 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>operational</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>retrofit</t>
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>45657</v>
+        <v>44561</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -5019,26 +5025,26 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>tata jlr</t>
+          <t>stellantis</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>halewood</t>
+          <t>tychy</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>halewood</t>
+          <t>tychy</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -5051,7 +5057,7 @@
         </is>
       </c>
       <c r="H47" s="2" t="n">
-        <v>43101</v>
+        <v>44927</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -5065,30 +5071,30 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Knowsley</t>
+          <t>Tychy</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Silesia</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Knowsley</t>
+          <t>Tychy</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Halewood</t>
+          <t>Tychy</t>
         </is>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
-        <v>53.36434</v>
+        <v>50.13717</v>
       </c>
       <c r="Q47" t="n">
-        <v>-2.82053</v>
+        <v>18.96641</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -5097,48 +5103,48 @@
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>29be1890-3777-517a-a337-0b7c8b408704</t>
+          <t>6d7b9e8a-1e97-5e07-8020-e277406f26cc</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_29be1890-3777-517a-a337-0b7c8b408704_20000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_6d7b9e8a-1e97-5e07-8020-e277406f26cc_40000.0</t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>GB|Knowsley|tata jlr|vehicle</t>
+          <t>PL|Tychy|stellantis|vehicle</t>
         </is>
       </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>('GB', 'Knowsley', 'tata jlr', 'vehicle')</t>
+          <t>('PL', 'Tychy', 'stellantis', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>tesla</t>
+          <t>stellantis</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>grünheide</t>
+          <t>tychy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>grünheide</t>
+          <t>tychy</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>320000</v>
+        <v>0</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -5147,11 +5153,11 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>greenfield</t>
+          <t>expansion</t>
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>44561</v>
+        <v>45658</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -5165,30 +5171,30 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Grünheide (Mark)</t>
+          <t>Tychy</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Brandenburg</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr"/>
+          <t>Silesia</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Tychy</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Landkreis Oder-Spree</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
-        <is>
-          <t>Grünheide (Mark)</t>
-        </is>
-      </c>
+          <t>Tychy</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>52.42343</v>
+        <v>50.13717</v>
       </c>
       <c r="Q48" t="n">
-        <v>13.81324</v>
+        <v>18.96641</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -5197,48 +5203,48 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>aa7e8a02-3dc6-59cf-bae6-5488cdc58c62</t>
+          <t>6d7b9e8a-1e97-5e07-8020-e277406f26cc</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_aa7e8a02-3dc6-59cf-bae6-5488cdc58c62_320000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_6d7b9e8a-1e97-5e07-8020-e277406f26cc_0.0</t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>DE|Grünheide (Mark)|tesla|vehicle</t>
+          <t>PL|Tychy|stellantis|vehicle</t>
         </is>
       </c>
       <c r="V48" t="inlineStr">
         <is>
-          <t>('DE', 'Grünheide (Mark)', 'tesla', 'vehicle')</t>
+          <t>('PL', 'Tychy', 'stellantis', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>tata jlr</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>hanover</t>
+          <t>halewood</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>hanover</t>
+          <t>halewood</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>40000</v>
+        <v>20000</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -5247,11 +5253,11 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>retrofit</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H49" s="2" t="n">
-        <v>44926</v>
+        <v>43101</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -5265,30 +5271,30 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Hanover</t>
+          <t>Knowsley</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Lower Saxony</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr"/>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Knowsley</t>
+        </is>
+      </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Region Hannover</t>
-        </is>
-      </c>
-      <c r="O49" t="inlineStr">
-        <is>
-          <t>Hanover</t>
-        </is>
-      </c>
+          <t>Halewood</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
-        <v>52.37052</v>
+        <v>53.36434</v>
       </c>
       <c r="Q49" t="n">
-        <v>9.733219999999999</v>
+        <v>-2.82053</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -5297,48 +5303,48 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>f50f1baf-752f-5614-a4b3-9dc9071ee0e9</t>
+          <t>29be1890-3777-517a-a337-0b7c8b408704</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_f50f1baf-752f-5614-a4b3-9dc9071ee0e9_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_29be1890-3777-517a-a337-0b7c8b408704_20000.0</t>
         </is>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>DE|Hanover|volkswagen|vehicle</t>
+          <t>GB|Knowsley|tata jlr|vehicle</t>
         </is>
       </c>
       <c r="V49" t="inlineStr">
         <is>
-          <t>('DE', 'Hanover', 'volkswagen', 'vehicle')</t>
+          <t>('GB', 'Knowsley', 'tata jlr', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>volkswagen</t>
+          <t>tesla</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>bratislava</t>
+          <t>grünheide</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>bratislava</t>
+          <t>grünheide</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>20000</v>
+        <v>320000</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -5351,7 +5357,7 @@
         </is>
       </c>
       <c r="H50" s="2" t="n">
-        <v>43830</v>
+        <v>44561</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -5365,22 +5371,30 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Bratislava Region</t>
+          <t>Grünheide (Mark)</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Bratislava Region</t>
+          <t>Brandenburg</t>
         </is>
       </c>
       <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-      <c r="O50" t="inlineStr"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Landkreis Oder-Spree</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Grünheide (Mark)</t>
+        </is>
+      </c>
       <c r="P50" t="n">
-        <v>48.14816</v>
+        <v>52.42343</v>
       </c>
       <c r="Q50" t="n">
-        <v>17.10674</v>
+        <v>13.81324</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -5389,22 +5403,22 @@
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>87caa632-7c5c-5e67-947b-59d0a19b7cd2</t>
+          <t>aa7e8a02-3dc6-59cf-bae6-5488cdc58c62</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_87caa632-7c5c-5e67-947b-59d0a19b7cd2_20000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_aa7e8a02-3dc6-59cf-bae6-5488cdc58c62_320000.0</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>SK|Bratislava Region|volkswagen|vehicle</t>
+          <t>DE|Grünheide (Mark)|tesla|vehicle</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>('SK', 'Bratislava Region', 'volkswagen', 'vehicle')</t>
+          <t>('DE', 'Grünheide (Mark)', 'tesla', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -5416,21 +5430,21 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>bratislava</t>
+          <t>hanover</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>bratislava</t>
+          <t>hanover</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>140000</v>
+        <v>40000</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -5439,11 +5453,11 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>expansion</t>
+          <t>retrofit</t>
         </is>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45291</v>
+        <v>44926</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -5457,22 +5471,30 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Bratislava Region</t>
+          <t>Hanover</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Bratislava Region</t>
+          <t>Lower Saxony</t>
         </is>
       </c>
       <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Region Hannover</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Hanover</t>
+        </is>
+      </c>
       <c r="P51" t="n">
-        <v>48.14816</v>
+        <v>52.37052</v>
       </c>
       <c r="Q51" t="n">
-        <v>17.10674</v>
+        <v>9.733219999999999</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -5481,48 +5503,48 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>87caa632-7c5c-5e67-947b-59d0a19b7cd2</t>
+          <t>f50f1baf-752f-5614-a4b3-9dc9071ee0e9</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_87caa632-7c5c-5e67-947b-59d0a19b7cd2_140000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_f50f1baf-752f-5614-a4b3-9dc9071ee0e9_40000.0</t>
         </is>
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>SK|Bratislava Region|volkswagen|vehicle</t>
+          <t>DE|Hanover|volkswagen|vehicle</t>
         </is>
       </c>
       <c r="V51" t="inlineStr">
         <is>
-          <t>('SK', 'Bratislava Region', 'volkswagen', 'vehicle')</t>
+          <t>('DE', 'Hanover', 'volkswagen', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>volvo</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>torslanda</t>
+          <t>bratislava</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>torslanda</t>
+          <t>bratislava</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>120000</v>
+        <v>20000</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -5531,11 +5553,11 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>greenfield</t>
         </is>
       </c>
       <c r="H52" s="2" t="n">
-        <v>45657</v>
+        <v>43830</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -5549,30 +5571,22 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Gothenburg Municipality</t>
+          <t>Bratislava Region</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Västra Götaland</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>Gothenburg Municipality</t>
-        </is>
-      </c>
-      <c r="N52" t="inlineStr">
-        <is>
-          <t>Torslanda</t>
-        </is>
-      </c>
+          <t>Bratislava Region</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
-        <v>57.72504</v>
+        <v>48.14816</v>
       </c>
       <c r="Q52" t="n">
-        <v>11.76903</v>
+        <v>17.10674</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
@@ -5581,48 +5595,48 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>018941f9-89ca-5292-bb96-95fcd1445d4f</t>
+          <t>87caa632-7c5c-5e67-947b-59d0a19b7cd2</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_018941f9-89ca-5292-bb96-95fcd1445d4f_120000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_87caa632-7c5c-5e67-947b-59d0a19b7cd2_20000.0</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>SE|Gothenburg Municipality|volvo|vehicle</t>
+          <t>SK|Bratislava Region|volkswagen|vehicle</t>
         </is>
       </c>
       <c r="V52" t="inlineStr">
         <is>
-          <t>('SE', 'Gothenburg Municipality', 'volvo', 'vehicle')</t>
+          <t>('SK', 'Bratislava Region', 'volkswagen', 'vehicle')</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>volvo</t>
+          <t>volkswagen</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ghent</t>
+          <t>bratislava</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ghent</t>
+          <t>bratislava</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>40000</v>
+        <v>140000</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -5631,11 +5645,11 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>greenfield</t>
+          <t>expansion</t>
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>44196</v>
+        <v>45291</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -5649,34 +5663,22 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Arrondissement of Ghent</t>
+          <t>Bratislava Region</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Flanders</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>East Flanders Province</t>
-        </is>
-      </c>
-      <c r="N53" t="inlineStr">
-        <is>
-          <t>Arrondissement of Ghent</t>
-        </is>
-      </c>
-      <c r="O53" t="inlineStr">
-        <is>
-          <t>Gent</t>
-        </is>
-      </c>
+          <t>Bratislava Region</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
       <c r="P53" t="n">
-        <v>51.05</v>
+        <v>48.14816</v>
       </c>
       <c r="Q53" t="n">
-        <v>3.71667</v>
+        <v>17.10674</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -5685,22 +5687,22 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>8727a516-7052-5f8b-a9da-0c21cb46ec42</t>
+          <t>87caa632-7c5c-5e67-947b-59d0a19b7cd2</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>68d684fc1c2e9d8ed1487afa_8727a516-7052-5f8b-a9da-0c21cb46ec42_40000.0</t>
+          <t>68d684fc1c2e9d8ed1487afa_87caa632-7c5c-5e67-947b-59d0a19b7cd2_140000.0</t>
         </is>
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>BE|Arrondissement of Ghent|volvo|vehicle</t>
+          <t>SK|Bratislava Region|volkswagen|vehicle</t>
         </is>
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>('BE', 'Arrondissement of Ghent', 'volvo', 'vehicle')</t>
+          <t>('SK', 'Bratislava Region', 'volkswagen', 'vehicle')</t>
         </is>
       </c>
     </row>
@@ -5712,21 +5714,21 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ghent</t>
+          <t>torslanda</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ghent</t>
+          <t>torslanda</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>200000</v>
+        <v>120000</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -5735,7 +5737,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>expansion</t>
+          <t>unclear</t>
         </is>
       </c>
       <c r="H54" s="2" t="n">
@@ -5753,56 +5755,260 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
+          <t>Gothenburg Municipality</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Västra Götaland</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Gothenburg Municipality</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Torslanda</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="n">
+        <v>57.72504</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>11.76903</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>68d684fc1c2e9d8ed1487afa</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>018941f9-89ca-5292-bb96-95fcd1445d4f</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>68d684fc1c2e9d8ed1487afa_018941f9-89ca-5292-bb96-95fcd1445d4f_120000.0</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>SE|Gothenburg Municipality|volvo|vehicle</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>('SE', 'Gothenburg Municipality', 'volvo', 'vehicle')</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>volvo</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ghent</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ghent</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>greenfield</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n">
+        <v>44196</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>vehicle</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>electric</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
           <t>Arrondissement of Ghent</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>Flanders</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>East Flanders Province</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>Arrondissement of Ghent</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>Gent</t>
         </is>
       </c>
-      <c r="P54" t="n">
+      <c r="P55" t="n">
         <v>51.05</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="Q55" t="n">
         <v>3.71667</v>
       </c>
-      <c r="R54" t="inlineStr">
+      <c r="R55" t="inlineStr">
         <is>
           <t>68d684fc1c2e9d8ed1487afa</t>
         </is>
       </c>
-      <c r="S54" t="inlineStr">
+      <c r="S55" t="inlineStr">
         <is>
           <t>8727a516-7052-5f8b-a9da-0c21cb46ec42</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr">
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>68d684fc1c2e9d8ed1487afa_8727a516-7052-5f8b-a9da-0c21cb46ec42_40000.0</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>BE|Arrondissement of Ghent|volvo|vehicle</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>('BE', 'Arrondissement of Ghent', 'volvo', 'vehicle')</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>volvo</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>ghent</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ghent</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>operational</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>expansion</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>45657</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>vehicle</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>electric</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Arrondissement of Ghent</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Flanders</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>East Flanders Province</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Arrondissement of Ghent</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Gent</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>51.05</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>3.71667</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>68d684fc1c2e9d8ed1487afa</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>8727a516-7052-5f8b-a9da-0c21cb46ec42</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
         <is>
           <t>68d684fc1c2e9d8ed1487afa_8727a516-7052-5f8b-a9da-0c21cb46ec42_200000.0</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>BE|Arrondissement of Ghent|volvo|vehicle</t>
         </is>
       </c>
-      <c r="V54" t="inlineStr">
+      <c r="V56" t="inlineStr">
         <is>
           <t>('BE', 'Arrondissement of Ghent', 'volvo', 'vehicle')</t>
         </is>

</xml_diff>